<commit_message>
4.5: Swine Manure (#202)
* feat(calculators): implemented chapter 4.5

* feat(calculators): re-implemented mnsoil calculation for swine manure and fixed tests

* chore: pr self-review

* chore: fixed example input
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/4.6-poultry-manure/4.6-poultry-manure.xlsx
+++ b/packages/calculators/src/modules/test/4.6-poultry-manure/4.6-poultry-manure.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11018"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mackcheesman/Desktop/Work/EAP/Code/emissions-calculators/packages/calculators/src/modules/test/4.6-poultry-manure/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19870AA3-BF9B-9143-9193-C594C696099E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FACA305F-99B4-AC45-BB86-63221D8D6F22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15860" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3775,15 +3775,15 @@
         <v>0.2</v>
       </c>
       <c r="V11">
-        <f>IF(F11="","",I11*J11/6.25)</f>
+        <f t="shared" ref="V11:V30" si="0">IF(F11="","",I11*J11/6.25)</f>
         <v>2.6144000000000002E-3</v>
       </c>
       <c r="W11">
-        <f>IF(F11="", "", V11*(1-K11))</f>
+        <f t="shared" ref="W11:W30" si="1">IF(F11="", "", V11*(1-K11))</f>
         <v>1.6993600000000002E-3</v>
       </c>
       <c r="X11">
-        <f>IF(F11="", "", G11*W11*H11)</f>
+        <f t="shared" ref="X11:X30" si="2">IF(F11="", "", G11*W11*H11)</f>
         <v>424.84000000000003</v>
       </c>
       <c r="Y11">
@@ -3791,11 +3791,11 @@
         <v>42.484000000000009</v>
       </c>
       <c r="Z11">
-        <f>IF(OR(L11="", L11="pastureRangeAndPaddock"), "", Y11*(1-R11-S11))</f>
+        <f t="shared" ref="Z11:Z30" si="3">IF(OR(L11="", L11="pastureRangeAndPaddock"), "", Y11*(1-R11-S11))</f>
         <v>29.69631600000001</v>
       </c>
       <c r="AA11">
-        <f>IF(F11="", "",SUM(Z11:Z15))</f>
+        <f t="shared" ref="AA11:AA30" si="4">IF(F11="", "",SUM(Z11:Z15))</f>
         <v>186.67469600000001</v>
       </c>
       <c r="AB11">
@@ -3811,11 +3811,11 @@
         <v>1.5714285714285714</v>
       </c>
       <c r="AE11">
-        <f>IF(L11="", "", Y11*R11*AD11)</f>
+        <f t="shared" ref="AE11:AE30" si="5">IF(L11="", "", Y11*R11*AD11)</f>
         <v>6.6760571428571433E-2</v>
       </c>
       <c r="AF11">
-        <f>IF(N11="directApplication", "", AB11*T11*AD11)</f>
+        <f t="shared" ref="AF11:AF30" si="6">IF(N11="directApplication", "", AB11*T11*AD11)</f>
         <v>0.22000946314285716</v>
       </c>
       <c r="AG11">
@@ -3823,7 +3823,7 @@
         <v>1.6022537142857147E-3</v>
       </c>
       <c r="AH11">
-        <f>IF(F11="","",SUM(AE11:AF15)/1000)</f>
+        <f t="shared" ref="AH11:AH30" si="7">IF(F11="","",SUM(AE11:AF15)/1000)</f>
         <v>6.5481105077142866E-3</v>
       </c>
       <c r="AI11">
@@ -3913,15 +3913,15 @@
         <v>0.2</v>
       </c>
       <c r="V12" t="str">
-        <f>IF(F12="","",I12*J12/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W12" t="str">
-        <f>IF(F12="", "", V12*(1-K12))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X12" t="str">
-        <f>IF(F12="", "", G12*W12*H12)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y12">
@@ -3929,11 +3929,11 @@
         <v>84.968000000000018</v>
       </c>
       <c r="Z12">
-        <f>IF(OR(L12="", L12="pastureRangeAndPaddock"), "", Y12*(1-R12-S12))</f>
+        <f t="shared" si="3"/>
         <v>80.634632000000011</v>
       </c>
       <c r="AA12" t="str">
-        <f>IF(F12="", "",SUM(Z12:Z16))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB12">
@@ -3949,11 +3949,11 @@
         <v>1.5714285714285714</v>
       </c>
       <c r="AE12">
-        <f>IF(L12="", "", Y12*R12*AD12)</f>
+        <f t="shared" si="5"/>
         <v>0.13352114285714287</v>
       </c>
       <c r="AF12">
-        <f>IF(N12="directApplication", "", AB12*T12*AD12)</f>
+        <f t="shared" si="6"/>
         <v>0.58669190171428576</v>
       </c>
       <c r="AG12" t="str">
@@ -3961,11 +3961,11 @@
         <v/>
       </c>
       <c r="AH12" t="str">
-        <f>IF(F12="","",SUM(AE12:AF16)/1000)</f>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="AI12" t="str">
-        <f t="shared" ref="AI12:AI30" si="0">IF(AG12="", "", AG12+AH12)</f>
+        <f t="shared" ref="AI12:AI30" si="8">IF(AG12="", "", AG12+AH12)</f>
         <v/>
       </c>
     </row>
@@ -4051,15 +4051,15 @@
         <v>0</v>
       </c>
       <c r="V13" t="str">
-        <f>IF(F13="","",I13*J13/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W13" t="str">
-        <f>IF(F13="", "", V13*(1-K13))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X13" t="str">
-        <f>IF(F13="", "", G13*W13*H13)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y13">
@@ -4067,11 +4067,11 @@
         <v>127.452</v>
       </c>
       <c r="Z13">
-        <f>IF(OR(L13="", L13="pastureRangeAndPaddock"), "", Y13*(1-R13-S13))</f>
+        <f t="shared" si="3"/>
         <v>76.343747999999991</v>
       </c>
       <c r="AA13" t="str">
-        <f>IF(F13="", "",SUM(Z13:Z17))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB13">
@@ -4087,11 +4087,11 @@
         <v>1.5714285714285714</v>
       </c>
       <c r="AE13">
-        <f>IF(L13="", "", Y13*R13*AD13)</f>
+        <f t="shared" si="5"/>
         <v>0.20028171428571429</v>
       </c>
       <c r="AF13">
-        <f>IF(N13="directApplication", "", AB13*T13*AD13)</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AG13" t="str">
@@ -4099,11 +4099,11 @@
         <v/>
       </c>
       <c r="AH13" t="str">
-        <f>IF(F13="","",SUM(AE13:AF17)/1000)</f>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="AI13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
@@ -4189,15 +4189,15 @@
         <v>0</v>
       </c>
       <c r="V14" t="str">
-        <f>IF(F14="","",I14*J14/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W14" t="str">
-        <f>IF(F14="", "", V14*(1-K14))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X14" t="str">
-        <f>IF(F14="", "", G14*W14*H14)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y14">
@@ -4205,11 +4205,11 @@
         <v>169.93600000000004</v>
       </c>
       <c r="Z14" t="str">
-        <f>IF(OR(L14="", L14="pastureRangeAndPaddock"), "", Y14*(1-R14-S14))</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA14" t="str">
-        <f>IF(F14="", "",SUM(Z14:Z18))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB14">
@@ -4225,11 +4225,11 @@
         <v>1.5714285714285714</v>
       </c>
       <c r="AE14">
-        <f>IF(L14="", "", Y14*R14*AD14)</f>
+        <f t="shared" si="5"/>
         <v>5.3408457142857158</v>
       </c>
       <c r="AF14">
-        <f>IF(N14="directApplication", "", AB14*T14*AD14)</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AG14" t="str">
@@ -4237,11 +4237,11 @@
         <v/>
       </c>
       <c r="AH14" t="str">
-        <f>IF(F14="","",SUM(AE14:AF18)/1000)</f>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="AI14" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
@@ -4321,15 +4321,15 @@
         <v>N/A</v>
       </c>
       <c r="V15" s="11" t="str">
-        <f>IF(F15="","",I15*J15/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W15" s="11" t="str">
-        <f>IF(F15="", "", V15*(1-K15))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X15" t="str">
-        <f>IF(F15="", "", G15*W15*H15)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y15" s="11" t="str">
@@ -4337,11 +4337,11 @@
         <v/>
       </c>
       <c r="Z15" t="str">
-        <f>IF(OR(L15="", L15="pastureRangeAndPaddock"), "", Y15*(1-R15-S15))</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA15" s="11" t="str">
-        <f>IF(F15="", "",SUM(Z15:Z19))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB15" t="str">
@@ -4357,11 +4357,11 @@
         <v>1.5714285714285714</v>
       </c>
       <c r="AE15" t="str">
-        <f>IF(L15="", "", Y15*R15*AD15)</f>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="AF15" t="str">
-        <f>IF(N15="directApplication", "", AB15*T15*AD15)</f>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AG15" t="str">
@@ -4369,11 +4369,11 @@
         <v/>
       </c>
       <c r="AH15" t="str">
-        <f>IF(F15="","",SUM(AE15:AF19)/1000)</f>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="AI15" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
@@ -4459,15 +4459,15 @@
         <v>0.2</v>
       </c>
       <c r="V16">
-        <f>IF(F16="","",I16*J16/6.25)</f>
+        <f t="shared" si="0"/>
         <v>3.1312000000000002E-3</v>
       </c>
       <c r="W16">
-        <f>IF(F16="", "", V16*(1-K16))</f>
+        <f t="shared" si="1"/>
         <v>2.1292159999999997E-3</v>
       </c>
       <c r="X16">
-        <f>IF(F16="", "", G16*W16*H16)</f>
+        <f t="shared" si="2"/>
         <v>598.84199999999987</v>
       </c>
       <c r="Y16">
@@ -4475,11 +4475,11 @@
         <v>239.53679999999997</v>
       </c>
       <c r="Z16">
-        <f>IF(OR(L16="", L16="pastureRangeAndPaddock"), "", Y16*(1-R16-S16))</f>
+        <f t="shared" si="3"/>
         <v>167.4362232</v>
       </c>
       <c r="AA16">
-        <f>IF(F16="", "",SUM(Z16:Z20))</f>
+        <f t="shared" si="4"/>
         <v>409.66781219999996</v>
       </c>
       <c r="AB16">
@@ -4495,11 +4495,11 @@
         <v>1.5714285714285714</v>
       </c>
       <c r="AE16">
-        <f>IF(L16="", "", Y16*R16*AD16)</f>
+        <f t="shared" si="5"/>
         <v>0.37641497142857139</v>
       </c>
       <c r="AF16">
-        <f>IF(N16="directApplication", "", AB16*T16*AD16)</f>
+        <f t="shared" si="6"/>
         <v>0.64376370488571433</v>
       </c>
       <c r="AG16">
@@ -4507,11 +4507,11 @@
         <v>1.8820748571428568E-4</v>
       </c>
       <c r="AH16">
-        <f>IF(F16="","",SUM(AE16:AF20)/1000)</f>
+        <f t="shared" si="7"/>
         <v>4.9821815099571429E-3</v>
       </c>
       <c r="AI16">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v>5.1703889956714287E-3</v>
       </c>
     </row>
@@ -4597,15 +4597,15 @@
         <v>0.2</v>
       </c>
       <c r="V17" t="str">
-        <f>IF(F17="","",I17*J17/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W17" t="str">
-        <f>IF(F17="", "", V17*(1-K17))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X17" t="str">
-        <f>IF(F17="", "", G17*W17*H17)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y17">
@@ -4613,11 +4613,11 @@
         <v>179.65259999999995</v>
       </c>
       <c r="Z17">
-        <f>IF(OR(L17="", L17="pastureRangeAndPaddock"), "", Y17*(1-R17-S17))</f>
+        <f t="shared" si="3"/>
         <v>170.49031739999995</v>
       </c>
       <c r="AA17" t="str">
-        <f>IF(F17="", "",SUM(Z17:Z21))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB17">
@@ -4633,11 +4633,11 @@
         <v>1.5714285714285714</v>
       </c>
       <c r="AE17">
-        <f>IF(L17="", "", Y17*R17*AD17)</f>
+        <f t="shared" si="5"/>
         <v>0.28231122857142849</v>
       </c>
       <c r="AF17">
-        <f>IF(N17="directApplication", "", AB17*T17*AD17)</f>
+        <f t="shared" si="6"/>
         <v>1.6094092622142855</v>
       </c>
       <c r="AG17" t="str">
@@ -4645,11 +4645,11 @@
         <v/>
       </c>
       <c r="AH17" t="str">
-        <f>IF(F17="","",SUM(AE17:AF21)/1000)</f>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="AI17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
@@ -4735,15 +4735,15 @@
         <v>0</v>
       </c>
       <c r="V18" t="str">
-        <f>IF(F18="","",I18*J18/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W18" t="str">
-        <f>IF(F18="", "", V18*(1-K18))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X18" t="str">
-        <f>IF(F18="", "", G18*W18*H18)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y18">
@@ -4751,11 +4751,11 @@
         <v>119.76839999999999</v>
       </c>
       <c r="Z18">
-        <f>IF(OR(L18="", L18="pastureRangeAndPaddock"), "", Y18*(1-R18-S18))</f>
+        <f t="shared" si="3"/>
         <v>71.74127159999999</v>
       </c>
       <c r="AA18" t="str">
-        <f>IF(F18="", "",SUM(Z18:Z22))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB18">
@@ -4771,11 +4771,11 @@
         <v>1.5714285714285714</v>
       </c>
       <c r="AE18">
-        <f>IF(L18="", "", Y18*R18*AD18)</f>
+        <f t="shared" si="5"/>
         <v>0.18820748571428569</v>
       </c>
       <c r="AF18">
-        <f>IF(N18="directApplication", "", AB18*T18*AD18)</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AG18" t="str">
@@ -4783,11 +4783,11 @@
         <v/>
       </c>
       <c r="AH18" t="str">
-        <f>IF(F18="","",SUM(AE18:AF22)/1000)</f>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="AI18" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
@@ -4873,15 +4873,15 @@
         <v>0</v>
       </c>
       <c r="V19" t="str">
-        <f>IF(F19="","",I19*J19/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W19" t="str">
-        <f>IF(F19="", "", V19*(1-K19))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X19" t="str">
-        <f>IF(F19="", "", G19*W19*H19)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y19">
@@ -4889,11 +4889,11 @@
         <v>59.884199999999993</v>
       </c>
       <c r="Z19" t="str">
-        <f>IF(OR(L19="", L19="pastureRangeAndPaddock"), "", Y19*(1-R19-S19))</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA19" t="str">
-        <f>IF(F19="", "",SUM(Z19:Z23))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB19">
@@ -4909,11 +4909,11 @@
         <v>1.5714285714285714</v>
       </c>
       <c r="AE19">
-        <f>IF(L19="", "", Y19*R19*AD19)</f>
+        <f t="shared" si="5"/>
         <v>1.8820748571428572</v>
       </c>
       <c r="AF19">
-        <f>IF(N19="directApplication", "", AB19*T19*AD19)</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AG19" t="str">
@@ -4921,11 +4921,11 @@
         <v/>
       </c>
       <c r="AH19" t="str">
-        <f>IF(F19="","",SUM(AE19:AF23)/1000)</f>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="AI19" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
@@ -5005,15 +5005,15 @@
         <v>N/A</v>
       </c>
       <c r="V20" s="11" t="str">
-        <f>IF(F20="","",I20*J20/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W20" s="11" t="str">
-        <f>IF(F20="", "", V20*(1-K20))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X20" t="str">
-        <f>IF(F20="", "", G20*W20*H20)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y20" s="11" t="str">
@@ -5021,11 +5021,11 @@
         <v/>
       </c>
       <c r="Z20" t="str">
-        <f>IF(OR(L20="", L20="pastureRangeAndPaddock"), "", Y20*(1-R20-S20))</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA20" s="11" t="str">
-        <f>IF(F20="", "",SUM(Z20:Z24))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB20" t="str">
@@ -5041,11 +5041,11 @@
         <v>1.5714285714285714</v>
       </c>
       <c r="AE20" t="str">
-        <f>IF(L20="", "", Y20*R20*AD20)</f>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="AF20" t="str">
-        <f>IF(N20="directApplication", "", AB20*T20*AD20)</f>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AG20" t="str">
@@ -5053,11 +5053,11 @@
         <v/>
       </c>
       <c r="AH20" t="str">
-        <f>IF(F20="","",SUM(AE20:AF24)/1000)</f>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="AI20" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
@@ -5143,15 +5143,15 @@
         <v>0.2</v>
       </c>
       <c r="V21">
-        <f>IF(F21="","",I21*J21/6.25)</f>
+        <f t="shared" si="0"/>
         <v>3.4223999999999999E-3</v>
       </c>
       <c r="W21">
-        <f>IF(F21="", "", V21*(1-K21))</f>
+        <f t="shared" si="1"/>
         <v>1.813872E-3</v>
       </c>
       <c r="X21">
-        <f>IF(F21="", "", G21*W21*H21)</f>
+        <f t="shared" si="2"/>
         <v>671.06552673600004</v>
       </c>
       <c r="Y21">
@@ -5159,11 +5159,11 @@
         <v>0</v>
       </c>
       <c r="Z21">
-        <f>IF(OR(L21="", L21="pastureRangeAndPaddock"), "", Y21*(1-R21-S21))</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AA21">
-        <f>IF(F21="", "",SUM(Z21:Z25))</f>
+        <f t="shared" si="4"/>
         <v>573.15706638521772</v>
       </c>
       <c r="AB21">
@@ -5179,11 +5179,11 @@
         <v>1.5714285714285714</v>
       </c>
       <c r="AE21">
-        <f>IF(L21="", "", Y21*R21*AD21)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AF21">
-        <f>IF(N21="directApplication", "", AB21*T21*AD21)</f>
+        <f t="shared" si="6"/>
         <v>1.5311481630576531</v>
       </c>
       <c r="AG21">
@@ -5191,11 +5191,11 @@
         <v>6.327189252082286E-4</v>
       </c>
       <c r="AH21">
-        <f>IF(F21="","",SUM(AE21:AF25)/1000)</f>
+        <f t="shared" si="7"/>
         <v>9.9933419751009056E-3</v>
       </c>
       <c r="AI21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v>1.0626060900309134E-2</v>
       </c>
     </row>
@@ -5281,15 +5281,15 @@
         <v>0.2</v>
       </c>
       <c r="V22" t="str">
-        <f>IF(F22="","",I22*J22/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W22" t="str">
-        <f>IF(F22="", "", V22*(1-K22))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X22" t="str">
-        <f>IF(F22="", "", G22*W22*H22)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y22">
@@ -5297,11 +5297,11 @@
         <v>603.9589740624001</v>
       </c>
       <c r="Z22">
-        <f>IF(OR(L22="", L22="pastureRangeAndPaddock"), "", Y22*(1-R22-S22))</f>
+        <f t="shared" si="3"/>
         <v>573.15706638521772</v>
       </c>
       <c r="AA22" t="str">
-        <f>IF(F22="", "",SUM(Z22:Z26))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB22">
@@ -5317,11 +5317,11 @@
         <v>1.5714285714285714</v>
       </c>
       <c r="AE22">
-        <f>IF(L22="", "", Y22*R22*AD22)</f>
+        <f t="shared" si="5"/>
         <v>0.94907838781234299</v>
       </c>
       <c r="AF22">
-        <f>IF(N22="directApplication", "", AB22*T22*AD22)</f>
+        <f t="shared" si="6"/>
         <v>5.4040523402034806</v>
       </c>
       <c r="AG22" t="str">
@@ -5329,11 +5329,11 @@
         <v/>
       </c>
       <c r="AH22" t="str">
-        <f>IF(F22="","",SUM(AE22:AF26)/1000)</f>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="AI22" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
@@ -5419,15 +5419,15 @@
         <v>0</v>
       </c>
       <c r="V23" t="str">
-        <f>IF(F23="","",I23*J23/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W23" t="str">
-        <f>IF(F23="", "", V23*(1-K23))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X23" t="str">
-        <f>IF(F23="", "", G23*W23*H23)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y23">
@@ -5435,11 +5435,11 @@
         <v>0</v>
       </c>
       <c r="Z23">
-        <f>IF(OR(L23="", L23="pastureRangeAndPaddock"), "", Y23*(1-R23-S23))</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AA23" t="str">
-        <f>IF(F23="", "",SUM(Z23:Z27))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB23">
@@ -5455,11 +5455,11 @@
         <v>1.5714285714285714</v>
       </c>
       <c r="AE23">
-        <f>IF(L23="", "", Y23*R23*AD23)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AF23">
-        <f>IF(N23="directApplication", "", AB23*T23*AD23)</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AG23" t="str">
@@ -5467,11 +5467,11 @@
         <v/>
       </c>
       <c r="AH23" t="str">
-        <f>IF(F23="","",SUM(AE23:AF27)/1000)</f>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="AI23" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
@@ -5557,15 +5557,15 @@
         <v>0</v>
       </c>
       <c r="V24" t="str">
-        <f>IF(F24="","",I24*J24/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W24" t="str">
-        <f>IF(F24="", "", V24*(1-K24))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X24" t="str">
-        <f>IF(F24="", "", G24*W24*H24)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y24">
@@ -5573,11 +5573,11 @@
         <v>67.106552673600007</v>
       </c>
       <c r="Z24" t="str">
-        <f>IF(OR(L24="", L24="pastureRangeAndPaddock"), "", Y24*(1-R24-S24))</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA24" t="str">
-        <f>IF(F24="", "",SUM(Z24:Z28))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB24">
@@ -5593,11 +5593,11 @@
         <v>1.5714285714285714</v>
       </c>
       <c r="AE24">
-        <f>IF(L24="", "", Y24*R24*AD24)</f>
+        <f t="shared" si="5"/>
         <v>2.1090630840274289</v>
       </c>
       <c r="AF24">
-        <f>IF(N24="directApplication", "", AB24*T24*AD24)</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AG24" t="str">
@@ -5605,11 +5605,11 @@
         <v/>
       </c>
       <c r="AH24" t="str">
-        <f>IF(F24="","",SUM(AE24:AF28)/1000)</f>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="AI24" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
@@ -5689,15 +5689,15 @@
         <v>N/A</v>
       </c>
       <c r="V25" s="11" t="str">
-        <f>IF(F25="","",I25*J25/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W25" s="11" t="str">
-        <f>IF(F25="", "", V25*(1-K25))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X25" t="str">
-        <f>IF(F25="", "", G25*W25*H25)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y25" s="11" t="str">
@@ -5705,11 +5705,11 @@
         <v/>
       </c>
       <c r="Z25" t="str">
-        <f>IF(OR(L25="", L25="pastureRangeAndPaddock"), "", Y25*(1-R25-S25))</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA25" s="11" t="str">
-        <f>IF(F25="", "",SUM(Z25:Z29))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB25" t="str">
@@ -5725,11 +5725,11 @@
         <v>1.5714285714285714</v>
       </c>
       <c r="AE25" t="str">
-        <f>IF(L25="", "", Y25*R25*AD25)</f>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="AF25" t="str">
-        <f>IF(N25="directApplication", "", AB25*T25*AD25)</f>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AG25" t="str">
@@ -5737,11 +5737,11 @@
         <v/>
       </c>
       <c r="AH25" t="str">
-        <f>IF(F25="","",SUM(AE25:AF29)/1000)</f>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="AI25" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
@@ -5827,15 +5827,15 @@
         <v>0.2</v>
       </c>
       <c r="V26">
-        <f>IF(F26="","",I26*J26/6.25)</f>
+        <f t="shared" si="0"/>
         <v>3.4223999999999999E-3</v>
       </c>
       <c r="W26">
-        <f>IF(F26="", "", V26*(1-K26))</f>
+        <f t="shared" si="1"/>
         <v>1.813872E-3</v>
       </c>
       <c r="X26">
-        <f>IF(F26="", "", G26*W26*H26)</f>
+        <f t="shared" si="2"/>
         <v>335.74770719999998</v>
       </c>
       <c r="Y26">
@@ -5843,11 +5843,11 @@
         <v>33.574770719999997</v>
       </c>
       <c r="Z26">
-        <f>IF(OR(L26="", L26="pastureRangeAndPaddock"), "", Y26*(1-R26-S26))</f>
+        <f t="shared" si="3"/>
         <v>23.46876473328</v>
       </c>
       <c r="AA26">
-        <f>IF(F26="", "",SUM(Z26:Z30))</f>
+        <f t="shared" si="4"/>
         <v>23.46876473328</v>
       </c>
       <c r="AB26">
@@ -5863,11 +5863,11 @@
         <v>1.5714285714285714</v>
       </c>
       <c r="AE26">
-        <f>IF(L26="", "", Y26*R26*AD26)</f>
+        <f t="shared" si="5"/>
         <v>5.2760353988571415E-2</v>
       </c>
       <c r="AF26">
-        <f>IF(N26="directApplication", "", AB26*T26*AD26)</f>
+        <f t="shared" si="6"/>
         <v>9.2198718595028567E-2</v>
       </c>
       <c r="AG26">
@@ -5875,11 +5875,11 @@
         <v>9.4968637179428561E-4</v>
       </c>
       <c r="AH26">
-        <f>IF(F26="","",SUM(AE26:AF30)/1000)</f>
+        <f t="shared" si="7"/>
         <v>9.7340215091214852E-3</v>
       </c>
       <c r="AI26">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v>1.0683707880915772E-2</v>
       </c>
     </row>
@@ -5965,15 +5965,15 @@
         <v>0.2</v>
       </c>
       <c r="V27" t="str">
-        <f>IF(F27="","",I27*J27/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W27" t="str">
-        <f>IF(F27="", "", V27*(1-K27))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X27" t="str">
-        <f>IF(F27="", "", G27*W27*H27)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y27">
@@ -5981,11 +5981,11 @@
         <v>0</v>
       </c>
       <c r="Z27">
-        <f>IF(OR(L27="", L27="pastureRangeAndPaddock"), "", Y27*(1-R27-S27))</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AA27" t="str">
-        <f>IF(F27="", "",SUM(Z27:Z31))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB27">
@@ -6001,11 +6001,11 @@
         <v>1.5714285714285714</v>
       </c>
       <c r="AE27">
-        <f>IF(L27="", "", Y27*R27*AD27)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AF27">
-        <f>IF(N27="directApplication", "", AB27*T27*AD27)</f>
+        <f t="shared" si="6"/>
         <v>9.2198718595028567E-2</v>
       </c>
       <c r="AG27" t="str">
@@ -6013,11 +6013,11 @@
         <v/>
       </c>
       <c r="AH27" t="str">
-        <f>IF(F27="","",SUM(AE27:AF31)/1000)</f>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="AI27" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
@@ -6103,15 +6103,15 @@
         <v>0</v>
       </c>
       <c r="V28" t="str">
-        <f>IF(F28="","",I28*J28/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W28" t="str">
-        <f>IF(F28="", "", V28*(1-K28))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X28" t="str">
-        <f>IF(F28="", "", G28*W28*H28)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y28">
@@ -6119,11 +6119,11 @@
         <v>0</v>
       </c>
       <c r="Z28">
-        <f>IF(OR(L28="", L28="pastureRangeAndPaddock"), "", Y28*(1-R28-S28))</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AA28" t="str">
-        <f>IF(F28="", "",SUM(Z28:Z32))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB28">
@@ -6139,11 +6139,11 @@
         <v>1.5714285714285714</v>
       </c>
       <c r="AE28">
-        <f>IF(L28="", "", Y28*R28*AD28)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AF28">
-        <f>IF(N28="directApplication", "", AB28*T28*AD28)</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AG28" t="str">
@@ -6151,11 +6151,11 @@
         <v/>
       </c>
       <c r="AH28" t="str">
-        <f>IF(F28="","",SUM(AE28:AF32)/1000)</f>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="AI28" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
@@ -6241,15 +6241,15 @@
         <v>0</v>
       </c>
       <c r="V29" t="str">
-        <f>IF(F29="","",I29*J29/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W29" t="str">
-        <f>IF(F29="", "", V29*(1-K29))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X29" t="str">
-        <f>IF(F29="", "", G29*W29*H29)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y29">
@@ -6257,11 +6257,11 @@
         <v>302.17293647999998</v>
       </c>
       <c r="Z29" t="str">
-        <f>IF(OR(L29="", L29="pastureRangeAndPaddock"), "", Y29*(1-R29-S29))</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA29" t="str">
-        <f>IF(F29="", "",SUM(Z29:Z33))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB29">
@@ -6277,11 +6277,11 @@
         <v>1.5714285714285714</v>
       </c>
       <c r="AE29">
-        <f>IF(L29="", "", Y29*R29*AD29)</f>
+        <f t="shared" si="5"/>
         <v>9.4968637179428566</v>
       </c>
       <c r="AF29">
-        <f>IF(N29="directApplication", "", AB29*T29*AD29)</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AG29" t="str">
@@ -6289,11 +6289,11 @@
         <v/>
       </c>
       <c r="AH29" t="str">
-        <f>IF(F29="","",SUM(AE29:AF33)/1000)</f>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="AI29" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
@@ -6373,15 +6373,15 @@
         <v>N/A</v>
       </c>
       <c r="V30" s="11" t="str">
-        <f>IF(F30="","",I30*J30/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W30" s="11" t="str">
-        <f>IF(F30="", "", V30*(1-K30))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X30" t="str">
-        <f>IF(F30="", "", G30*W30*H30)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y30" s="11" t="str">
@@ -6389,11 +6389,11 @@
         <v/>
       </c>
       <c r="Z30" t="str">
-        <f>IF(OR(L30="", L30="pastureRangeAndPaddock"), "", Y30*(1-R30-S30))</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA30" s="11" t="str">
-        <f>IF(F30="", "",SUM(Z30:Z34))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB30" t="str">
@@ -6409,11 +6409,11 @@
         <v>1.5714285714285714</v>
       </c>
       <c r="AE30" t="str">
-        <f>IF(L30="", "", Y30*R30*AD30)</f>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="AF30" t="str">
-        <f>IF(N30="directApplication", "", AB30*T30*AD30)</f>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AG30" t="str">
@@ -6421,11 +6421,11 @@
         <v/>
       </c>
       <c r="AH30" t="str">
-        <f>IF(F30="","",SUM(AE30:AF34)/1000)</f>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="AI30" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
@@ -6781,15 +6781,15 @@
         <v>0.2</v>
       </c>
       <c r="V11">
-        <f>IF(F11="","",I11*J11/6.25)</f>
+        <f t="shared" ref="V11:V30" si="0">IF(F11="","",I11*J11/6.25)</f>
         <v>2.6144000000000002E-3</v>
       </c>
       <c r="W11">
-        <f>IF(F11="", "", V11*(1-K11))</f>
+        <f t="shared" ref="W11:W30" si="1">IF(F11="", "", V11*(1-K11))</f>
         <v>1.6993600000000002E-3</v>
       </c>
       <c r="X11">
-        <f>IF(F11="", "", G11*W11*H11)</f>
+        <f t="shared" ref="X11:X30" si="2">IF(F11="", "", G11*W11*H11)</f>
         <v>424.84000000000003</v>
       </c>
       <c r="Y11">
@@ -6797,11 +6797,11 @@
         <v>42.484000000000009</v>
       </c>
       <c r="Z11">
-        <f>IF(OR(L11="", L11="pastureRangeAndPaddock"), "", Y11*(1-R11-S11))</f>
+        <f t="shared" ref="Z11:Z30" si="3">IF(OR(L11="", L11="pastureRangeAndPaddock"), "", Y11*(1-R11-S11))</f>
         <v>29.69631600000001</v>
       </c>
       <c r="AA11">
-        <f>IF(F11="", "",SUM(Z11:Z15))</f>
+        <f t="shared" ref="AA11:AA30" si="4">IF(F11="", "",SUM(Z11:Z15))</f>
         <v>186.67469600000001</v>
       </c>
       <c r="AB11">
@@ -6813,11 +6813,11 @@
         <v>12.745200000000002</v>
       </c>
       <c r="AD11">
-        <f>IF(OR(N11="", N11="directApplication"), "",AB11*U11)</f>
+        <f t="shared" ref="AD11:AD30" si="5">IF(OR(N11="", N11="directApplication"), "",AB11*U11)</f>
         <v>5.6002408800000012</v>
       </c>
       <c r="AE11">
-        <f>IF(F11="", "", SUM(AC11:AD15))</f>
+        <f t="shared" ref="AE11:AE30" si="6">IF(F11="", "", SUM(AC11:AD15))</f>
         <v>116.72818872000002</v>
       </c>
       <c r="AF11">
@@ -6915,15 +6915,15 @@
         <v>0.2</v>
       </c>
       <c r="V12" t="str">
-        <f>IF(F12="","",I12*J12/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W12" t="str">
-        <f>IF(F12="", "", V12*(1-K12))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X12" t="str">
-        <f>IF(F12="", "", G12*W12*H12)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y12">
@@ -6931,11 +6931,11 @@
         <v>84.968000000000018</v>
       </c>
       <c r="Z12">
-        <f>IF(OR(L12="", L12="pastureRangeAndPaddock"), "", Y12*(1-R12-S12))</f>
+        <f t="shared" si="3"/>
         <v>80.634632000000011</v>
       </c>
       <c r="AA12" t="str">
-        <f>IF(F12="", "",SUM(Z12:Z16))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB12">
@@ -6947,11 +6947,11 @@
         <v>4.2484000000000011</v>
       </c>
       <c r="AD12">
-        <f>IF(OR(N12="", N12="directApplication"), "",AB12*U12)</f>
+        <f t="shared" si="5"/>
         <v>7.4669878400000007</v>
       </c>
       <c r="AE12" t="str">
-        <f>IF(F12="", "", SUM(AC12:AD16))</f>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AF12" t="str">
@@ -6963,7 +6963,7 @@
         <v/>
       </c>
       <c r="AH12" t="str">
-        <f t="shared" ref="AH12:AH30" si="0">IF(AE12="", "", (AE12*AF12*AG12)/1000)</f>
+        <f t="shared" ref="AH12:AH30" si="7">IF(AE12="", "", (AE12*AF12*AG12)/1000)</f>
         <v/>
       </c>
     </row>
@@ -7049,15 +7049,15 @@
         <v>0</v>
       </c>
       <c r="V13" t="str">
-        <f>IF(F13="","",I13*J13/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W13" t="str">
-        <f>IF(F13="", "", V13*(1-K13))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X13" t="str">
-        <f>IF(F13="", "", G13*W13*H13)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y13">
@@ -7065,11 +7065,11 @@
         <v>127.452</v>
       </c>
       <c r="Z13">
-        <f>IF(OR(L13="", L13="pastureRangeAndPaddock"), "", Y13*(1-R13-S13))</f>
+        <f t="shared" si="3"/>
         <v>76.343747999999991</v>
       </c>
       <c r="AA13" t="str">
-        <f>IF(F13="", "",SUM(Z13:Z17))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB13">
@@ -7081,11 +7081,11 @@
         <v>50.980800000000002</v>
       </c>
       <c r="AD13">
-        <f>IF(OR(N13="", N13="directApplication"), "",AB13*U13)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AE13" t="str">
-        <f>IF(F13="", "", SUM(AC13:AD17))</f>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AF13" t="str">
@@ -7097,7 +7097,7 @@
         <v/>
       </c>
       <c r="AH13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
@@ -7183,15 +7183,15 @@
         <v>0</v>
       </c>
       <c r="V14" t="str">
-        <f>IF(F14="","",I14*J14/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W14" t="str">
-        <f>IF(F14="", "", V14*(1-K14))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X14" t="str">
-        <f>IF(F14="", "", G14*W14*H14)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y14">
@@ -7199,11 +7199,11 @@
         <v>169.93600000000004</v>
       </c>
       <c r="Z14" t="str">
-        <f>IF(OR(L14="", L14="pastureRangeAndPaddock"), "", Y14*(1-R14-S14))</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA14" t="str">
-        <f>IF(F14="", "",SUM(Z14:Z18))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB14">
@@ -7215,11 +7215,11 @@
         <v>35.686560000000007</v>
       </c>
       <c r="AD14">
-        <f>IF(OR(N14="", N14="directApplication"), "",AB14*U14)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AE14" t="str">
-        <f>IF(F14="", "", SUM(AC14:AD18))</f>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AF14" t="str">
@@ -7231,7 +7231,7 @@
         <v/>
       </c>
       <c r="AH14" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
@@ -7311,15 +7311,15 @@
         <v>N/A</v>
       </c>
       <c r="V15" s="11" t="str">
-        <f>IF(F15="","",I15*J15/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W15" s="11" t="str">
-        <f>IF(F15="", "", V15*(1-K15))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X15" t="str">
-        <f>IF(F15="", "", G15*W15*H15)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y15" s="11" t="str">
@@ -7327,11 +7327,11 @@
         <v/>
       </c>
       <c r="Z15" t="str">
-        <f>IF(OR(L15="", L15="pastureRangeAndPaddock"), "", Y15*(1-R15-S15))</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA15" s="11" t="str">
-        <f>IF(F15="", "",SUM(Z15:Z19))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB15" t="str">
@@ -7343,11 +7343,11 @@
         <v/>
       </c>
       <c r="AD15" t="str">
-        <f>IF(OR(N15="", N15="directApplication"), "",AB15*U15)</f>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="AE15" t="str">
-        <f>IF(F15="", "", SUM(AC15:AD19))</f>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AF15" t="str">
@@ -7359,7 +7359,7 @@
         <v/>
       </c>
       <c r="AH15" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
@@ -7445,15 +7445,15 @@
         <v>0.2</v>
       </c>
       <c r="V16">
-        <f>IF(F16="","",I16*J16/6.25)</f>
+        <f t="shared" si="0"/>
         <v>3.1312000000000002E-3</v>
       </c>
       <c r="W16">
-        <f>IF(F16="", "", V16*(1-K16))</f>
+        <f t="shared" si="1"/>
         <v>2.1292159999999997E-3</v>
       </c>
       <c r="X16">
-        <f>IF(F16="", "", G16*W16*H16)</f>
+        <f t="shared" si="2"/>
         <v>598.84199999999987</v>
       </c>
       <c r="Y16">
@@ -7461,11 +7461,11 @@
         <v>239.53679999999997</v>
       </c>
       <c r="Z16">
-        <f>IF(OR(L16="", L16="pastureRangeAndPaddock"), "", Y16*(1-R16-S16))</f>
+        <f t="shared" si="3"/>
         <v>167.4362232</v>
       </c>
       <c r="AA16">
-        <f>IF(F16="", "",SUM(Z16:Z20))</f>
+        <f t="shared" si="4"/>
         <v>409.66781219999996</v>
       </c>
       <c r="AB16">
@@ -7477,11 +7477,11 @@
         <v>71.861039999999988</v>
       </c>
       <c r="AD16">
-        <f>IF(OR(N16="", N16="directApplication"), "",AB16*U16)</f>
+        <f t="shared" si="5"/>
         <v>16.386712488000001</v>
       </c>
       <c r="AE16">
-        <f>IF(F16="", "", SUM(AC16:AD20))</f>
+        <f t="shared" si="6"/>
         <v>178.19681509799997</v>
       </c>
       <c r="AF16">
@@ -7493,7 +7493,7 @@
         <v>1.5714285714285714</v>
       </c>
       <c r="AH16">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>1.9601649660779996E-3</v>
       </c>
     </row>
@@ -7579,15 +7579,15 @@
         <v>0.2</v>
       </c>
       <c r="V17" t="str">
-        <f>IF(F17="","",I17*J17/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W17" t="str">
-        <f>IF(F17="", "", V17*(1-K17))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X17" t="str">
-        <f>IF(F17="", "", G17*W17*H17)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y17">
@@ -7595,11 +7595,11 @@
         <v>179.65259999999995</v>
       </c>
       <c r="Z17">
-        <f>IF(OR(L17="", L17="pastureRangeAndPaddock"), "", Y17*(1-R17-S17))</f>
+        <f t="shared" si="3"/>
         <v>170.49031739999995</v>
       </c>
       <c r="AA17" t="str">
-        <f>IF(F17="", "",SUM(Z17:Z21))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB17">
@@ -7611,11 +7611,11 @@
         <v>8.9826299999999986</v>
       </c>
       <c r="AD17">
-        <f>IF(OR(N17="", N17="directApplication"), "",AB17*U17)</f>
+        <f t="shared" si="5"/>
         <v>20.483390610000001</v>
       </c>
       <c r="AE17" t="str">
-        <f>IF(F17="", "", SUM(AC17:AD21))</f>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AF17" t="str">
@@ -7627,7 +7627,7 @@
         <v/>
       </c>
       <c r="AH17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
@@ -7713,15 +7713,15 @@
         <v>0</v>
       </c>
       <c r="V18" t="str">
-        <f>IF(F18="","",I18*J18/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W18" t="str">
-        <f>IF(F18="", "", V18*(1-K18))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X18" t="str">
-        <f>IF(F18="", "", G18*W18*H18)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y18">
@@ -7729,11 +7729,11 @@
         <v>119.76839999999999</v>
       </c>
       <c r="Z18">
-        <f>IF(OR(L18="", L18="pastureRangeAndPaddock"), "", Y18*(1-R18-S18))</f>
+        <f t="shared" si="3"/>
         <v>71.74127159999999</v>
       </c>
       <c r="AA18" t="str">
-        <f>IF(F18="", "",SUM(Z18:Z22))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB18">
@@ -7745,11 +7745,11 @@
         <v>47.907359999999997</v>
       </c>
       <c r="AD18">
-        <f>IF(OR(N18="", N18="directApplication"), "",AB18*U18)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AE18" t="str">
-        <f>IF(F18="", "", SUM(AC18:AD22))</f>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AF18" t="str">
@@ -7761,7 +7761,7 @@
         <v/>
       </c>
       <c r="AH18" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
@@ -7847,15 +7847,15 @@
         <v>0</v>
       </c>
       <c r="V19" t="str">
-        <f>IF(F19="","",I19*J19/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W19" t="str">
-        <f>IF(F19="", "", V19*(1-K19))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X19" t="str">
-        <f>IF(F19="", "", G19*W19*H19)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y19">
@@ -7863,11 +7863,11 @@
         <v>59.884199999999993</v>
       </c>
       <c r="Z19" t="str">
-        <f>IF(OR(L19="", L19="pastureRangeAndPaddock"), "", Y19*(1-R19-S19))</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA19" t="str">
-        <f>IF(F19="", "",SUM(Z19:Z23))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB19">
@@ -7879,11 +7879,11 @@
         <v>12.575681999999999</v>
       </c>
       <c r="AD19">
-        <f>IF(OR(N19="", N19="directApplication"), "",AB19*U19)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AE19" t="str">
-        <f>IF(F19="", "", SUM(AC19:AD23))</f>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AF19" t="str">
@@ -7895,7 +7895,7 @@
         <v/>
       </c>
       <c r="AH19" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
@@ -7975,15 +7975,15 @@
         <v>N/A</v>
       </c>
       <c r="V20" s="11" t="str">
-        <f>IF(F20="","",I20*J20/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W20" s="11" t="str">
-        <f>IF(F20="", "", V20*(1-K20))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X20" t="str">
-        <f>IF(F20="", "", G20*W20*H20)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y20" s="11" t="str">
@@ -7991,11 +7991,11 @@
         <v/>
       </c>
       <c r="Z20" t="str">
-        <f>IF(OR(L20="", L20="pastureRangeAndPaddock"), "", Y20*(1-R20-S20))</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA20" s="11" t="str">
-        <f>IF(F20="", "",SUM(Z20:Z24))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB20" t="str">
@@ -8007,11 +8007,11 @@
         <v/>
       </c>
       <c r="AD20" t="str">
-        <f>IF(OR(N20="", N20="directApplication"), "",AB20*U20)</f>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="AE20" t="str">
-        <f>IF(F20="", "", SUM(AC20:AD24))</f>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AF20" t="str">
@@ -8023,7 +8023,7 @@
         <v/>
       </c>
       <c r="AH20" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
@@ -8109,15 +8109,15 @@
         <v>0.2</v>
       </c>
       <c r="V21">
-        <f>IF(F21="","",I21*J21/6.25)</f>
+        <f t="shared" si="0"/>
         <v>3.4223999999999999E-3</v>
       </c>
       <c r="W21">
-        <f>IF(F21="", "", V21*(1-K21))</f>
+        <f t="shared" si="1"/>
         <v>1.813872E-3</v>
       </c>
       <c r="X21">
-        <f>IF(F21="", "", G21*W21*H21)</f>
+        <f t="shared" si="2"/>
         <v>671.06552673600004</v>
       </c>
       <c r="Y21">
@@ -8125,11 +8125,11 @@
         <v>0</v>
       </c>
       <c r="Z21">
-        <f>IF(OR(L21="", L21="pastureRangeAndPaddock"), "", Y21*(1-R21-S21))</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AA21">
-        <f>IF(F21="", "",SUM(Z21:Z25))</f>
+        <f t="shared" si="4"/>
         <v>573.15706638521772</v>
       </c>
       <c r="AB21">
@@ -8141,11 +8141,11 @@
         <v>0</v>
       </c>
       <c r="AD21">
-        <f>IF(OR(N21="", N21="directApplication"), "",AB21*U21)</f>
+        <f t="shared" si="5"/>
         <v>38.974680514194809</v>
       </c>
       <c r="AE21">
-        <f>IF(F21="", "", SUM(AC21:AD25))</f>
+        <f t="shared" si="6"/>
         <v>152.04385324499694</v>
       </c>
       <c r="AF21">
@@ -8157,7 +8157,7 @@
         <v>1.5714285714285714</v>
       </c>
       <c r="AH21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>1.4096637250857571E-3</v>
       </c>
     </row>
@@ -8243,15 +8243,15 @@
         <v>0.2</v>
       </c>
       <c r="V22" t="str">
-        <f>IF(F22="","",I22*J22/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W22" t="str">
-        <f>IF(F22="", "", V22*(1-K22))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X22" t="str">
-        <f>IF(F22="", "", G22*W22*H22)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y22">
@@ -8259,11 +8259,11 @@
         <v>603.9589740624001</v>
       </c>
       <c r="Z22">
-        <f>IF(OR(L22="", L22="pastureRangeAndPaddock"), "", Y22*(1-R22-S22))</f>
+        <f t="shared" si="3"/>
         <v>573.15706638521772</v>
       </c>
       <c r="AA22" t="str">
-        <f>IF(F22="", "",SUM(Z22:Z26))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB22">
@@ -8275,11 +8275,11 @@
         <v>30.197948703120005</v>
       </c>
       <c r="AD22">
-        <f>IF(OR(N22="", N22="directApplication"), "",AB22*U22)</f>
+        <f t="shared" si="5"/>
         <v>68.778847966226124</v>
       </c>
       <c r="AE22" t="str">
-        <f>IF(F22="", "", SUM(AC22:AD26))</f>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AF22" t="str">
@@ -8291,7 +8291,7 @@
         <v/>
       </c>
       <c r="AH22" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
@@ -8377,15 +8377,15 @@
         <v>0</v>
       </c>
       <c r="V23" t="str">
-        <f>IF(F23="","",I23*J23/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W23" t="str">
-        <f>IF(F23="", "", V23*(1-K23))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X23" t="str">
-        <f>IF(F23="", "", G23*W23*H23)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y23">
@@ -8393,11 +8393,11 @@
         <v>0</v>
       </c>
       <c r="Z23">
-        <f>IF(OR(L23="", L23="pastureRangeAndPaddock"), "", Y23*(1-R23-S23))</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AA23" t="str">
-        <f>IF(F23="", "",SUM(Z23:Z27))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB23">
@@ -8409,11 +8409,11 @@
         <v>0</v>
       </c>
       <c r="AD23">
-        <f>IF(OR(N23="", N23="directApplication"), "",AB23*U23)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AE23" t="str">
-        <f>IF(F23="", "", SUM(AC23:AD27))</f>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AF23" t="str">
@@ -8425,7 +8425,7 @@
         <v/>
       </c>
       <c r="AH23" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
@@ -8511,15 +8511,15 @@
         <v>0</v>
       </c>
       <c r="V24" t="str">
-        <f>IF(F24="","",I24*J24/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W24" t="str">
-        <f>IF(F24="", "", V24*(1-K24))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X24" t="str">
-        <f>IF(F24="", "", G24*W24*H24)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y24">
@@ -8527,11 +8527,11 @@
         <v>67.106552673600007</v>
       </c>
       <c r="Z24" t="str">
-        <f>IF(OR(L24="", L24="pastureRangeAndPaddock"), "", Y24*(1-R24-S24))</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA24" t="str">
-        <f>IF(F24="", "",SUM(Z24:Z28))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB24">
@@ -8543,11 +8543,11 @@
         <v>14.092376061456001</v>
       </c>
       <c r="AD24">
-        <f>IF(OR(N24="", N24="directApplication"), "",AB24*U24)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AE24" t="str">
-        <f>IF(F24="", "", SUM(AC24:AD28))</f>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AF24" t="str">
@@ -8559,7 +8559,7 @@
         <v/>
       </c>
       <c r="AH24" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
@@ -8639,15 +8639,15 @@
         <v>N/A</v>
       </c>
       <c r="V25" s="11" t="str">
-        <f>IF(F25="","",I25*J25/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W25" s="11" t="str">
-        <f>IF(F25="", "", V25*(1-K25))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X25" t="str">
-        <f>IF(F25="", "", G25*W25*H25)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y25" s="11" t="str">
@@ -8655,11 +8655,11 @@
         <v/>
       </c>
       <c r="Z25" t="str">
-        <f>IF(OR(L25="", L25="pastureRangeAndPaddock"), "", Y25*(1-R25-S25))</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA25" s="11" t="str">
-        <f>IF(F25="", "",SUM(Z25:Z29))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB25" t="str">
@@ -8671,11 +8671,11 @@
         <v/>
       </c>
       <c r="AD25" t="str">
-        <f>IF(OR(N25="", N25="directApplication"), "",AB25*U25)</f>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="AE25" t="str">
-        <f>IF(F25="", "", SUM(AC25:AD29))</f>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AF25" t="str">
@@ -8687,7 +8687,7 @@
         <v/>
       </c>
       <c r="AH25" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
@@ -8773,15 +8773,15 @@
         <v>0.2</v>
       </c>
       <c r="V26">
-        <f>IF(F26="","",I26*J26/6.25)</f>
+        <f t="shared" si="0"/>
         <v>3.4223999999999999E-3</v>
       </c>
       <c r="W26">
-        <f>IF(F26="", "", V26*(1-K26))</f>
+        <f t="shared" si="1"/>
         <v>1.813872E-3</v>
       </c>
       <c r="X26">
-        <f>IF(F26="", "", G26*W26*H26)</f>
+        <f t="shared" si="2"/>
         <v>335.74770719999998</v>
       </c>
       <c r="Y26">
@@ -8789,11 +8789,11 @@
         <v>33.574770719999997</v>
       </c>
       <c r="Z26">
-        <f>IF(OR(L26="", L26="pastureRangeAndPaddock"), "", Y26*(1-R26-S26))</f>
+        <f t="shared" si="3"/>
         <v>23.46876473328</v>
       </c>
       <c r="AA26">
-        <f>IF(F26="", "",SUM(Z26:Z30))</f>
+        <f t="shared" si="4"/>
         <v>23.46876473328</v>
       </c>
       <c r="AB26">
@@ -8805,11 +8805,11 @@
         <v>10.072431215999998</v>
       </c>
       <c r="AD26">
-        <f>IF(OR(N26="", N26="directApplication"), "",AB26*U26)</f>
+        <f t="shared" si="5"/>
         <v>2.3468764733280003</v>
       </c>
       <c r="AE26">
-        <f>IF(F26="", "", SUM(AC26:AD30))</f>
+        <f t="shared" si="6"/>
         <v>77.04906258679199</v>
       </c>
       <c r="AF26">
@@ -8821,7 +8821,7 @@
         <v>1.5714285714285714</v>
       </c>
       <c r="AH26">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>9.68616786805385E-4</v>
       </c>
     </row>
@@ -8907,15 +8907,15 @@
         <v>0.2</v>
       </c>
       <c r="V27" t="str">
-        <f>IF(F27="","",I27*J27/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W27" t="str">
-        <f>IF(F27="", "", V27*(1-K27))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X27" t="str">
-        <f>IF(F27="", "", G27*W27*H27)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y27">
@@ -8923,11 +8923,11 @@
         <v>0</v>
       </c>
       <c r="Z27">
-        <f>IF(OR(L27="", L27="pastureRangeAndPaddock"), "", Y27*(1-R27-S27))</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AA27" t="str">
-        <f>IF(F27="", "",SUM(Z27:Z31))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB27">
@@ -8939,11 +8939,11 @@
         <v>0</v>
       </c>
       <c r="AD27">
-        <f>IF(OR(N27="", N27="directApplication"), "",AB27*U27)</f>
+        <f t="shared" si="5"/>
         <v>1.1734382366640002</v>
       </c>
       <c r="AE27" t="str">
-        <f>IF(F27="", "", SUM(AC27:AD31))</f>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AF27" t="str">
@@ -8955,7 +8955,7 @@
         <v/>
       </c>
       <c r="AH27" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
@@ -9041,15 +9041,15 @@
         <v>0</v>
       </c>
       <c r="V28" t="str">
-        <f>IF(F28="","",I28*J28/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W28" t="str">
-        <f>IF(F28="", "", V28*(1-K28))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X28" t="str">
-        <f>IF(F28="", "", G28*W28*H28)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y28">
@@ -9057,11 +9057,11 @@
         <v>0</v>
       </c>
       <c r="Z28">
-        <f>IF(OR(L28="", L28="pastureRangeAndPaddock"), "", Y28*(1-R28-S28))</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AA28" t="str">
-        <f>IF(F28="", "",SUM(Z28:Z32))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB28">
@@ -9073,11 +9073,11 @@
         <v>0</v>
       </c>
       <c r="AD28">
-        <f>IF(OR(N28="", N28="directApplication"), "",AB28*U28)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AE28" t="str">
-        <f>IF(F28="", "", SUM(AC28:AD32))</f>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AF28" t="str">
@@ -9089,7 +9089,7 @@
         <v/>
       </c>
       <c r="AH28" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
@@ -9175,15 +9175,15 @@
         <v>0</v>
       </c>
       <c r="V29" t="str">
-        <f>IF(F29="","",I29*J29/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W29" t="str">
-        <f>IF(F29="", "", V29*(1-K29))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X29" t="str">
-        <f>IF(F29="", "", G29*W29*H29)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y29">
@@ -9191,11 +9191,11 @@
         <v>302.17293647999998</v>
       </c>
       <c r="Z29" t="str">
-        <f>IF(OR(L29="", L29="pastureRangeAndPaddock"), "", Y29*(1-R29-S29))</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA29" t="str">
-        <f>IF(F29="", "",SUM(Z29:Z33))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB29">
@@ -9207,11 +9207,11 @@
         <v>63.456316660799992</v>
       </c>
       <c r="AD29">
-        <f>IF(OR(N29="", N29="directApplication"), "",AB29*U29)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AE29" t="str">
-        <f>IF(F29="", "", SUM(AC29:AD33))</f>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AF29" t="str">
@@ -9223,7 +9223,7 @@
         <v/>
       </c>
       <c r="AH29" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
@@ -9303,15 +9303,15 @@
         <v>N/A</v>
       </c>
       <c r="V30" s="11" t="str">
-        <f>IF(F30="","",I30*J30/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W30" s="11" t="str">
-        <f>IF(F30="", "", V30*(1-K30))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X30" t="str">
-        <f>IF(F30="", "", G30*W30*H30)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y30" s="11" t="str">
@@ -9319,11 +9319,11 @@
         <v/>
       </c>
       <c r="Z30" t="str">
-        <f>IF(OR(L30="", L30="pastureRangeAndPaddock"), "", Y30*(1-R30-S30))</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA30" s="11" t="str">
-        <f>IF(F30="", "",SUM(Z30:Z34))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB30" t="str">
@@ -9335,11 +9335,11 @@
         <v/>
       </c>
       <c r="AD30" t="str">
-        <f>IF(OR(N30="", N30="directApplication"), "",AB30*U30)</f>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="AE30" t="str">
-        <f>IF(F30="", "", SUM(AC30:AD34))</f>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AF30" t="str">
@@ -9351,7 +9351,7 @@
         <v/>
       </c>
       <c r="AH30" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
@@ -9709,15 +9709,15 @@
         <v>0.2</v>
       </c>
       <c r="V11">
-        <f>IF(F11="","",I11*J11/6.25)</f>
+        <f t="shared" ref="V11:V30" si="0">IF(F11="","",I11*J11/6.25)</f>
         <v>2.6144000000000002E-3</v>
       </c>
       <c r="W11">
-        <f>IF(F11="", "", V11*(1-K11))</f>
+        <f t="shared" ref="W11:W30" si="1">IF(F11="", "", V11*(1-K11))</f>
         <v>1.6993600000000002E-3</v>
       </c>
       <c r="X11">
-        <f>IF(F11="", "", G11*W11*H11)</f>
+        <f t="shared" ref="X11:X30" si="2">IF(F11="", "", G11*W11*H11)</f>
         <v>424.84000000000003</v>
       </c>
       <c r="Y11">
@@ -9725,11 +9725,11 @@
         <v>42.484000000000009</v>
       </c>
       <c r="Z11">
-        <f>IF(OR(L11="", L11="pastureRangeAndPaddock"), "", Y11*(1-R11-S11))</f>
+        <f t="shared" ref="Z11:Z30" si="3">IF(OR(L11="", L11="pastureRangeAndPaddock"), "", Y11*(1-R11-S11))</f>
         <v>29.69631600000001</v>
       </c>
       <c r="AA11">
-        <f>IF(F11="", "",SUM(Z11:Z15))</f>
+        <f t="shared" ref="AA11:AA30" si="4">IF(F11="", "",SUM(Z11:Z15))</f>
         <v>186.67469600000001</v>
       </c>
       <c r="AB11">
@@ -9847,15 +9847,15 @@
         <v>0.2</v>
       </c>
       <c r="V12" t="str">
-        <f>IF(F12="","",I12*J12/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W12" t="str">
-        <f>IF(F12="", "", V12*(1-K12))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X12" t="str">
-        <f>IF(F12="", "", G12*W12*H12)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y12">
@@ -9863,11 +9863,11 @@
         <v>84.968000000000018</v>
       </c>
       <c r="Z12">
-        <f>IF(OR(L12="", L12="pastureRangeAndPaddock"), "", Y12*(1-R12-S12))</f>
+        <f t="shared" si="3"/>
         <v>80.634632000000011</v>
       </c>
       <c r="AA12" t="str">
-        <f>IF(F12="", "",SUM(Z12:Z16))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB12">
@@ -9875,7 +9875,7 @@
         <v>37.334939200000001</v>
       </c>
       <c r="AC12" t="str">
-        <f t="shared" ref="AC12:AC30" si="0">IF(E12="", "", IF(E12, 1, 0))</f>
+        <f t="shared" ref="AC12:AC30" si="5">IF(E12="", "", IF(E12, 1, 0))</f>
         <v/>
       </c>
       <c r="AD12" t="str">
@@ -9891,15 +9891,15 @@
         <v/>
       </c>
       <c r="AG12" t="str">
-        <f t="shared" ref="AG12:AG30" si="1">IF(N12="solidStorage", AB12*AC12*AD12, "")</f>
+        <f t="shared" ref="AG12:AG30" si="6">IF(N12="solidStorage", AB12*AC12*AD12, "")</f>
         <v/>
       </c>
       <c r="AH12" t="str">
-        <f t="shared" ref="AH12:AH30" si="2">IF(L15="pastureRangeAndPaddock", Y15*AD$11*AC$11, "")</f>
+        <f t="shared" ref="AH12:AH15" si="7">IF(L15="pastureRangeAndPaddock", Y15*AD$11*AC$11, "")</f>
         <v/>
       </c>
       <c r="AI12" t="str">
-        <f t="shared" ref="AI12:AI31" si="3">IF(F12="", "", (AG12+AH12)*AE12*AF12/1000)</f>
+        <f t="shared" ref="AI12:AI31" si="8">IF(F12="", "", (AG12+AH12)*AE12*AF12/1000)</f>
         <v/>
       </c>
     </row>
@@ -9985,15 +9985,15 @@
         <v>0</v>
       </c>
       <c r="V13" t="str">
-        <f>IF(F13="","",I13*J13/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W13" t="str">
-        <f>IF(F13="", "", V13*(1-K13))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X13" t="str">
-        <f>IF(F13="", "", G13*W13*H13)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y13">
@@ -10001,11 +10001,11 @@
         <v>127.452</v>
       </c>
       <c r="Z13">
-        <f>IF(OR(L13="", L13="pastureRangeAndPaddock"), "", Y13*(1-R13-S13))</f>
+        <f t="shared" si="3"/>
         <v>76.343747999999991</v>
       </c>
       <c r="AA13" t="str">
-        <f>IF(F13="", "",SUM(Z13:Z17))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB13">
@@ -10013,7 +10013,7 @@
         <v>46.668674000000003</v>
       </c>
       <c r="AC13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="AD13" t="str">
@@ -10029,15 +10029,15 @@
         <v/>
       </c>
       <c r="AG13" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AH13" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="AI13" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
@@ -10123,15 +10123,15 @@
         <v>0</v>
       </c>
       <c r="V14" t="str">
-        <f>IF(F14="","",I14*J14/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W14" t="str">
-        <f>IF(F14="", "", V14*(1-K14))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X14" t="str">
-        <f>IF(F14="", "", G14*W14*H14)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y14">
@@ -10139,11 +10139,11 @@
         <v>169.93600000000004</v>
       </c>
       <c r="Z14" t="str">
-        <f>IF(OR(L14="", L14="pastureRangeAndPaddock"), "", Y14*(1-R14-S14))</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA14" t="str">
-        <f>IF(F14="", "",SUM(Z14:Z18))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB14">
@@ -10151,7 +10151,7 @@
         <v>31.734698320000003</v>
       </c>
       <c r="AC14" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="AD14" t="str">
@@ -10167,15 +10167,15 @@
         <v/>
       </c>
       <c r="AG14" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AH14" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="AI14" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
@@ -10255,15 +10255,15 @@
         <v>N/A</v>
       </c>
       <c r="V15" s="11" t="str">
-        <f>IF(F15="","",I15*J15/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W15" s="11" t="str">
-        <f>IF(F15="", "", V15*(1-K15))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X15" t="str">
-        <f>IF(F15="", "", G15*W15*H15)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y15" s="11" t="str">
@@ -10271,11 +10271,11 @@
         <v/>
       </c>
       <c r="Z15" t="str">
-        <f>IF(OR(L15="", L15="pastureRangeAndPaddock"), "", Y15*(1-R15-S15))</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA15" s="11" t="str">
-        <f>IF(F15="", "",SUM(Z15:Z19))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB15" t="str">
@@ -10283,7 +10283,7 @@
         <v/>
       </c>
       <c r="AC15" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="AD15" t="str">
@@ -10299,15 +10299,15 @@
         <v/>
       </c>
       <c r="AG15" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AH15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="AI15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
@@ -10329,8 +10329,7 @@
         <v>dry</v>
       </c>
       <c r="E16" t="b">
-        <f>IF(ISBLANK('Input Scenarios'!E13), "", 'Input Scenarios'!E13)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F16" t="str">
         <f>IF(ISBLANK('Input Scenarios'!F13), "", 'Input Scenarios'!F13)</f>
@@ -10393,15 +10392,15 @@
         <v>0.2</v>
       </c>
       <c r="V16">
-        <f>IF(F16="","",I16*J16/6.25)</f>
+        <f t="shared" si="0"/>
         <v>3.1312000000000002E-3</v>
       </c>
       <c r="W16">
-        <f>IF(F16="", "", V16*(1-K16))</f>
+        <f t="shared" si="1"/>
         <v>2.1292159999999997E-3</v>
       </c>
       <c r="X16">
-        <f>IF(F16="", "", G16*W16*H16)</f>
+        <f t="shared" si="2"/>
         <v>598.84199999999987</v>
       </c>
       <c r="Y16">
@@ -10409,11 +10408,11 @@
         <v>239.53679999999997</v>
       </c>
       <c r="Z16">
-        <f>IF(OR(L16="", L16="pastureRangeAndPaddock"), "", Y16*(1-R16-S16))</f>
+        <f t="shared" si="3"/>
         <v>167.4362232</v>
       </c>
       <c r="AA16">
-        <f>IF(F16="", "",SUM(Z16:Z20))</f>
+        <f t="shared" si="4"/>
         <v>409.66781219999996</v>
       </c>
       <c r="AB16">
@@ -10421,8 +10420,8 @@
         <v>81.933562440000003</v>
       </c>
       <c r="AC16">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="5"/>
+        <v>0</v>
       </c>
       <c r="AD16">
         <f>IF(E16="","",Constants!$M$2)</f>
@@ -10437,16 +10436,16 @@
         <v>1.5714285714285714</v>
       </c>
       <c r="AG16">
-        <f t="shared" si="1"/>
-        <v>1.6386712488000001</v>
+        <f t="shared" si="6"/>
+        <v>0</v>
       </c>
       <c r="AH16">
         <f>IF(L19="pastureRangeAndPaddock", Y19*AD$16*AC$16, "")</f>
-        <v>1.197684</v>
+        <v>0</v>
       </c>
       <c r="AI16">
-        <f t="shared" si="3"/>
-        <v>4.9028426443542864E-5</v>
+        <f t="shared" si="8"/>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:35" x14ac:dyDescent="0.2">
@@ -10531,15 +10530,15 @@
         <v>0.2</v>
       </c>
       <c r="V17" t="str">
-        <f>IF(F17="","",I17*J17/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W17" t="str">
-        <f>IF(F17="", "", V17*(1-K17))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X17" t="str">
-        <f>IF(F17="", "", G17*W17*H17)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y17">
@@ -10547,11 +10546,11 @@
         <v>179.65259999999995</v>
       </c>
       <c r="Z17">
-        <f>IF(OR(L17="", L17="pastureRangeAndPaddock"), "", Y17*(1-R17-S17))</f>
+        <f t="shared" si="3"/>
         <v>170.49031739999995</v>
       </c>
       <c r="AA17" t="str">
-        <f>IF(F17="", "",SUM(Z17:Z21))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB17">
@@ -10559,7 +10558,7 @@
         <v>102.41695304999999</v>
       </c>
       <c r="AC17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="AD17" t="str">
@@ -10575,15 +10574,15 @@
         <v/>
       </c>
       <c r="AG17" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AH17" t="str">
-        <f t="shared" ref="AH17:AH20" si="4">IF(L20="pastureRangeAndPaddock", Y20*AD$16*AC$16, "")</f>
+        <f t="shared" ref="AH17:AH20" si="9">IF(L20="pastureRangeAndPaddock", Y20*AD$16*AC$16, "")</f>
         <v/>
       </c>
       <c r="AI17" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
@@ -10669,15 +10668,15 @@
         <v>0</v>
       </c>
       <c r="V18" t="str">
-        <f>IF(F18="","",I18*J18/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W18" t="str">
-        <f>IF(F18="", "", V18*(1-K18))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X18" t="str">
-        <f>IF(F18="", "", G18*W18*H18)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y18">
@@ -10685,11 +10684,11 @@
         <v>119.76839999999999</v>
       </c>
       <c r="Z18">
-        <f>IF(OR(L18="", L18="pastureRangeAndPaddock"), "", Y18*(1-R18-S18))</f>
+        <f t="shared" si="3"/>
         <v>71.74127159999999</v>
       </c>
       <c r="AA18" t="str">
-        <f>IF(F18="", "",SUM(Z18:Z22))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB18">
@@ -10697,7 +10696,7 @@
         <v>81.933562440000003</v>
       </c>
       <c r="AC18" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="AD18" t="str">
@@ -10713,15 +10712,15 @@
         <v/>
       </c>
       <c r="AG18" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AH18" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="AI18" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
@@ -10807,15 +10806,15 @@
         <v>0</v>
       </c>
       <c r="V19" t="str">
-        <f>IF(F19="","",I19*J19/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W19" t="str">
-        <f>IF(F19="", "", V19*(1-K19))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X19" t="str">
-        <f>IF(F19="", "", G19*W19*H19)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y19">
@@ -10823,11 +10822,11 @@
         <v>59.884199999999993</v>
       </c>
       <c r="Z19" t="str">
-        <f>IF(OR(L19="", L19="pastureRangeAndPaddock"), "", Y19*(1-R19-S19))</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA19" t="str">
-        <f>IF(F19="", "",SUM(Z19:Z23))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB19">
@@ -10835,7 +10834,7 @@
         <v>102.41695304999999</v>
       </c>
       <c r="AC19" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="AD19" t="str">
@@ -10851,15 +10850,15 @@
         <v/>
       </c>
       <c r="AG19" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AH19" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="AI19" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
@@ -10939,15 +10938,15 @@
         <v>N/A</v>
       </c>
       <c r="V20" s="11" t="str">
-        <f>IF(F20="","",I20*J20/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W20" s="11" t="str">
-        <f>IF(F20="", "", V20*(1-K20))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X20" t="str">
-        <f>IF(F20="", "", G20*W20*H20)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y20" s="11" t="str">
@@ -10955,11 +10954,11 @@
         <v/>
       </c>
       <c r="Z20" t="str">
-        <f>IF(OR(L20="", L20="pastureRangeAndPaddock"), "", Y20*(1-R20-S20))</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA20" s="11" t="str">
-        <f>IF(F20="", "",SUM(Z20:Z24))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB20" t="str">
@@ -10967,7 +10966,7 @@
         <v/>
       </c>
       <c r="AC20" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="AD20" t="str">
@@ -10983,15 +10982,15 @@
         <v/>
       </c>
       <c r="AG20" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AH20" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="AI20" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
@@ -11077,15 +11076,15 @@
         <v>0.2</v>
       </c>
       <c r="V21">
-        <f>IF(F21="","",I21*J21/6.25)</f>
+        <f t="shared" si="0"/>
         <v>3.4223999999999999E-3</v>
       </c>
       <c r="W21">
-        <f>IF(F21="", "", V21*(1-K21))</f>
+        <f t="shared" si="1"/>
         <v>1.813872E-3</v>
       </c>
       <c r="X21">
-        <f>IF(F21="", "", G21*W21*H21)</f>
+        <f t="shared" si="2"/>
         <v>671.06552673600004</v>
       </c>
       <c r="Y21">
@@ -11093,11 +11092,11 @@
         <v>0</v>
       </c>
       <c r="Z21">
-        <f>IF(OR(L21="", L21="pastureRangeAndPaddock"), "", Y21*(1-R21-S21))</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AA21">
-        <f>IF(F21="", "",SUM(Z21:Z25))</f>
+        <f t="shared" si="4"/>
         <v>573.15706638521772</v>
       </c>
       <c r="AB21">
@@ -11105,7 +11104,7 @@
         <v>194.87340257097404</v>
       </c>
       <c r="AC21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AD21">
@@ -11121,7 +11120,7 @@
         <v>1.5714285714285714</v>
       </c>
       <c r="AG21">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>3.8974680514194806</v>
       </c>
       <c r="AH21">
@@ -11129,7 +11128,7 @@
         <v>1.3421310534720001</v>
       </c>
       <c r="AI21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>9.0570213098838429E-5</v>
       </c>
     </row>
@@ -11215,15 +11214,15 @@
         <v>0.2</v>
       </c>
       <c r="V22" t="str">
-        <f>IF(F22="","",I22*J22/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W22" t="str">
-        <f>IF(F22="", "", V22*(1-K22))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X22" t="str">
-        <f>IF(F22="", "", G22*W22*H22)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y22">
@@ -11231,11 +11230,11 @@
         <v>603.9589740624001</v>
       </c>
       <c r="Z22">
-        <f>IF(OR(L22="", L22="pastureRangeAndPaddock"), "", Y22*(1-R22-S22))</f>
+        <f t="shared" si="3"/>
         <v>573.15706638521772</v>
       </c>
       <c r="AA22" t="str">
-        <f>IF(F22="", "",SUM(Z22:Z26))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB22">
@@ -11243,7 +11242,7 @@
         <v>343.89423983113062</v>
       </c>
       <c r="AC22" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="AD22" t="str">
@@ -11259,15 +11258,15 @@
         <v/>
       </c>
       <c r="AG22" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AH22" t="str">
-        <f t="shared" ref="AH22:AH30" si="5">IF(L25="pastureRangeAndPaddock", Y25*AD$21*AC$21, "")</f>
+        <f t="shared" ref="AH22:AH25" si="10">IF(L25="pastureRangeAndPaddock", Y25*AD$21*AC$21, "")</f>
         <v/>
       </c>
       <c r="AI22" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
@@ -11353,15 +11352,15 @@
         <v>0</v>
       </c>
       <c r="V23" t="str">
-        <f>IF(F23="","",I23*J23/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W23" t="str">
-        <f>IF(F23="", "", V23*(1-K23))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X23" t="str">
-        <f>IF(F23="", "", G23*W23*H23)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y23">
@@ -11369,11 +11368,11 @@
         <v>0</v>
       </c>
       <c r="Z23">
-        <f>IF(OR(L23="", L23="pastureRangeAndPaddock"), "", Y23*(1-R23-S23))</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AA23" t="str">
-        <f>IF(F23="", "",SUM(Z23:Z27))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB23">
@@ -11381,7 +11380,7 @@
         <v>0</v>
       </c>
       <c r="AC23" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="AD23" t="str">
@@ -11397,15 +11396,15 @@
         <v/>
       </c>
       <c r="AG23" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AH23" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="AI23" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
@@ -11491,15 +11490,15 @@
         <v>0</v>
       </c>
       <c r="V24" t="str">
-        <f>IF(F24="","",I24*J24/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W24" t="str">
-        <f>IF(F24="", "", V24*(1-K24))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X24" t="str">
-        <f>IF(F24="", "", G24*W24*H24)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y24">
@@ -11507,11 +11506,11 @@
         <v>67.106552673600007</v>
       </c>
       <c r="Z24" t="str">
-        <f>IF(OR(L24="", L24="pastureRangeAndPaddock"), "", Y24*(1-R24-S24))</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA24" t="str">
-        <f>IF(F24="", "",SUM(Z24:Z28))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB24">
@@ -11519,7 +11518,7 @@
         <v>0</v>
       </c>
       <c r="AC24" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="AD24" t="str">
@@ -11535,15 +11534,15 @@
         <v/>
       </c>
       <c r="AG24" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AH24" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="AI24" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
@@ -11623,15 +11622,15 @@
         <v>N/A</v>
       </c>
       <c r="V25" s="11" t="str">
-        <f>IF(F25="","",I25*J25/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W25" s="11" t="str">
-        <f>IF(F25="", "", V25*(1-K25))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X25" t="str">
-        <f>IF(F25="", "", G25*W25*H25)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y25" s="11" t="str">
@@ -11639,11 +11638,11 @@
         <v/>
       </c>
       <c r="Z25" t="str">
-        <f>IF(OR(L25="", L25="pastureRangeAndPaddock"), "", Y25*(1-R25-S25))</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA25" s="11" t="str">
-        <f>IF(F25="", "",SUM(Z25:Z29))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB25" t="str">
@@ -11651,7 +11650,7 @@
         <v/>
       </c>
       <c r="AC25" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="AD25" t="str">
@@ -11667,15 +11666,15 @@
         <v/>
       </c>
       <c r="AG25" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AH25" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="AI25" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
@@ -11761,15 +11760,15 @@
         <v>0.2</v>
       </c>
       <c r="V26">
-        <f>IF(F26="","",I26*J26/6.25)</f>
+        <f t="shared" si="0"/>
         <v>3.4223999999999999E-3</v>
       </c>
       <c r="W26">
-        <f>IF(F26="", "", V26*(1-K26))</f>
+        <f t="shared" si="1"/>
         <v>1.813872E-3</v>
       </c>
       <c r="X26">
-        <f>IF(F26="", "", G26*W26*H26)</f>
+        <f t="shared" si="2"/>
         <v>335.74770719999998</v>
       </c>
       <c r="Y26">
@@ -11777,11 +11776,11 @@
         <v>33.574770719999997</v>
       </c>
       <c r="Z26">
-        <f>IF(OR(L26="", L26="pastureRangeAndPaddock"), "", Y26*(1-R26-S26))</f>
+        <f t="shared" si="3"/>
         <v>23.46876473328</v>
       </c>
       <c r="AA26">
-        <f>IF(F26="", "",SUM(Z26:Z30))</f>
+        <f t="shared" si="4"/>
         <v>23.46876473328</v>
       </c>
       <c r="AB26">
@@ -11789,7 +11788,7 @@
         <v>11.73438236664</v>
       </c>
       <c r="AC26">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AD26">
@@ -11805,7 +11804,7 @@
         <v>1.5714285714285714</v>
       </c>
       <c r="AG26">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>0.23468764733280001</v>
       </c>
       <c r="AH26">
@@ -11813,7 +11812,7 @@
         <v>6.0434587295999993</v>
       </c>
       <c r="AI26">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>1.0852224451555266E-4</v>
       </c>
     </row>
@@ -11899,15 +11898,15 @@
         <v>0.2</v>
       </c>
       <c r="V27" t="str">
-        <f>IF(F27="","",I27*J27/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W27" t="str">
-        <f>IF(F27="", "", V27*(1-K27))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X27" t="str">
-        <f>IF(F27="", "", G27*W27*H27)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y27">
@@ -11915,11 +11914,11 @@
         <v>0</v>
       </c>
       <c r="Z27">
-        <f>IF(OR(L27="", L27="pastureRangeAndPaddock"), "", Y27*(1-R27-S27))</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AA27" t="str">
-        <f>IF(F27="", "",SUM(Z27:Z31))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB27">
@@ -11927,7 +11926,7 @@
         <v>5.8671911833200001</v>
       </c>
       <c r="AC27" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="AD27" t="str">
@@ -11943,15 +11942,15 @@
         <v/>
       </c>
       <c r="AG27" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AH27" t="str">
-        <f t="shared" ref="AH27:AH30" si="6">IF(L30="pastureRangeAndPaddock", Y30*AD$26*AC$26, "")</f>
+        <f t="shared" ref="AH27:AH30" si="11">IF(L30="pastureRangeAndPaddock", Y30*AD$26*AC$26, "")</f>
         <v/>
       </c>
       <c r="AI27" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
@@ -12037,15 +12036,15 @@
         <v>0</v>
       </c>
       <c r="V28" t="str">
-        <f>IF(F28="","",I28*J28/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W28" t="str">
-        <f>IF(F28="", "", V28*(1-K28))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X28" t="str">
-        <f>IF(F28="", "", G28*W28*H28)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y28">
@@ -12053,11 +12052,11 @@
         <v>0</v>
       </c>
       <c r="Z28">
-        <f>IF(OR(L28="", L28="pastureRangeAndPaddock"), "", Y28*(1-R28-S28))</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AA28" t="str">
-        <f>IF(F28="", "",SUM(Z28:Z32))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB28">
@@ -12065,7 +12064,7 @@
         <v>5.8671911833200001</v>
       </c>
       <c r="AC28" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="AD28" t="str">
@@ -12081,15 +12080,15 @@
         <v/>
       </c>
       <c r="AG28" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AH28" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="AI28" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
@@ -12175,15 +12174,15 @@
         <v>0</v>
       </c>
       <c r="V29" t="str">
-        <f>IF(F29="","",I29*J29/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W29" t="str">
-        <f>IF(F29="", "", V29*(1-K29))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X29" t="str">
-        <f>IF(F29="", "", G29*W29*H29)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y29">
@@ -12191,11 +12190,11 @@
         <v>302.17293647999998</v>
       </c>
       <c r="Z29" t="str">
-        <f>IF(OR(L29="", L29="pastureRangeAndPaddock"), "", Y29*(1-R29-S29))</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA29" t="str">
-        <f>IF(F29="", "",SUM(Z29:Z33))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB29">
@@ -12203,7 +12202,7 @@
         <v>0</v>
       </c>
       <c r="AC29" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="AD29" t="str">
@@ -12219,15 +12218,15 @@
         <v/>
       </c>
       <c r="AG29" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AH29" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="AI29" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
@@ -12307,15 +12306,15 @@
         <v>N/A</v>
       </c>
       <c r="V30" s="11" t="str">
-        <f>IF(F30="","",I30*J30/6.25)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="W30" s="11" t="str">
-        <f>IF(F30="", "", V30*(1-K30))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X30" t="str">
-        <f>IF(F30="", "", G30*W30*H30)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Y30" s="11" t="str">
@@ -12323,11 +12322,11 @@
         <v/>
       </c>
       <c r="Z30" t="str">
-        <f>IF(OR(L30="", L30="pastureRangeAndPaddock"), "", Y30*(1-R30-S30))</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA30" s="11" t="str">
-        <f>IF(F30="", "",SUM(Z30:Z34))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AB30" t="str">
@@ -12335,7 +12334,7 @@
         <v/>
       </c>
       <c r="AC30" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="AD30" t="str">
@@ -12351,21 +12350,21 @@
         <v/>
       </c>
       <c r="AG30" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AH30" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="AI30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="31" spans="1:35" x14ac:dyDescent="0.2">
       <c r="AI31" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: forgot to commit changes to test spreadsheet
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/4.6-poultry-manure/4.6-poultry-manure.xlsx
+++ b/packages/calculators/src/modules/test/4.6-poultry-manure/4.6-poultry-manure.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mackcheesman/Desktop/Work/EAP/Code/emissions-calculators/packages/calculators/src/modules/test/4.6-poultry-manure/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B9D7B04-2C32-654C-8AC6-66D76C6D2E45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E67F5B8-FC51-954F-8452-B5E9FE41C329}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-6820" yWindow="-21600" windowWidth="38400" windowHeight="21600" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="4.6.1.1" sheetId="5" r:id="rId1"/>
@@ -8050,7 +8050,7 @@
       <c r="BQ10" s="14" t="s">
         <v>210</v>
       </c>
-      <c r="BR10" s="14" t="s">
+      <c r="BR10" s="15" t="s">
         <v>85</v>
       </c>
       <c r="BS10" s="15" t="s">
@@ -9490,7 +9490,7 @@
         <v>6.9011177039999989</v>
       </c>
       <c r="BS15" s="12">
-        <f t="shared" si="9"/>
+        <f>AU15+BR15</f>
         <v>12.941883863999998</v>
       </c>
       <c r="BT15">

</xml_diff>